<commit_message>
Wire in official InXpress logos (white in app header, blue on reports)
- Commit official PNG logos under assets/brand/media
- brand.logo_path(on_dark) returns brand-correct logo per background
- Streamlit header shows white logo (base64) on Midnight Blue; wordmark fallback
- Excel reports show blue logo on white above the title band
- 34 tests passing; app serves HTTP 200; reports regenerated with logo

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/sample-customer-report.xlsx
+++ b/reports/sample-customer-report.xlsx
@@ -181,6 +181,36 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="390525"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -472,7 +502,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F148"/>
+  <dimension ref="A2:F149"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -483,126 +513,103 @@
     <col width="9" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="34" customHeight="1"/>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>Freight IQ — Your savings summary</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="16" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
+    <row r="3" ht="16" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>InXpress Edmonton &amp; Atlantic Canada  |  platinumsupport@inxpress.com  |  902 706 7666</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Target customer savings: 15%</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>Summary</t>
         </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>Shipments reviewed</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="n">
-        <v>481</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>Lanes we can save you on</t>
+          <t>Shipments reviewed</t>
         </is>
       </c>
       <c r="B8" s="4" t="n">
-        <v>137</v>
+        <v>481</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
+          <t>Lanes we can save you on</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="n">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
           <t>Total estimated savings</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>$1,051.38</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="6" t="inlineStr">
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="6" t="inlineStr">
         <is>
           <t>Tracking</t>
         </is>
       </c>
-      <c r="B11" s="6" t="inlineStr">
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>Service</t>
         </is>
       </c>
-      <c r="C11" s="6" t="inlineStr">
+      <c r="C12" s="6" t="inlineStr">
         <is>
           <t>Current price</t>
         </is>
       </c>
-      <c r="D11" s="6" t="inlineStr">
+      <c r="D12" s="6" t="inlineStr">
         <is>
           <t>Your InXpress price</t>
         </is>
       </c>
-      <c r="E11" s="6" t="inlineStr">
+      <c r="E12" s="6" t="inlineStr">
         <is>
           <t>You save</t>
         </is>
       </c>
-      <c r="F11" s="6" t="inlineStr">
+      <c r="F12" s="6" t="inlineStr">
         <is>
           <t>% saved</t>
         </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>1ZE88F612057631095</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Standard</t>
-        </is>
-      </c>
-      <c r="C12" s="7" t="n">
-        <v>27.43</v>
-      </c>
-      <c r="D12" s="7" t="n">
-        <v>27.21</v>
-      </c>
-      <c r="E12" s="8" t="n">
-        <v>0.22</v>
-      </c>
-      <c r="F12" s="9" t="n">
-        <v>0.008020415603353991</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>1ZE88F612056200463</t>
+          <t>1ZE88F612057631095</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -611,142 +618,142 @@
         </is>
       </c>
       <c r="C13" s="7" t="n">
-        <v>29.46</v>
+        <v>27.43</v>
       </c>
       <c r="D13" s="7" t="n">
-        <v>29.46</v>
+        <v>27.21</v>
       </c>
       <c r="E13" s="8" t="n">
-        <v>0</v>
+        <v>0.22</v>
       </c>
       <c r="F13" s="9" t="n">
-        <v>0</v>
+        <v>0.008020415603353991</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>1ZE88F611455561613</t>
+          <t>1ZE88F612056200463</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Express</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="C14" s="7" t="n">
-        <v>35.12</v>
+        <v>29.46</v>
       </c>
       <c r="D14" s="7" t="n">
-        <v>30.27</v>
+        <v>29.46</v>
       </c>
       <c r="E14" s="8" t="n">
-        <v>4.85</v>
+        <v>0</v>
       </c>
       <c r="F14" s="9" t="n">
-        <v>0.1380979498861048</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>1ZE88F612057109641</t>
+          <t>1ZE88F611455561613</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Express</t>
         </is>
       </c>
       <c r="C15" s="7" t="n">
-        <v>20.67</v>
+        <v>35.12</v>
       </c>
       <c r="D15" s="7" t="n">
-        <v>17.57</v>
+        <v>30.27</v>
       </c>
       <c r="E15" s="8" t="n">
-        <v>3.1</v>
+        <v>4.85</v>
       </c>
       <c r="F15" s="9" t="n">
-        <v>0.1499758103531688</v>
+        <v>0.1380979498861048</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>1ZE88F611457362389</t>
+          <t>1ZE88F612057109641</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Express</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="C16" s="7" t="n">
-        <v>35.12</v>
+        <v>20.67</v>
       </c>
       <c r="D16" s="7" t="n">
-        <v>30.27</v>
+        <v>17.57</v>
       </c>
       <c r="E16" s="8" t="n">
-        <v>4.85</v>
+        <v>3.1</v>
       </c>
       <c r="F16" s="9" t="n">
-        <v>0.1380979498861048</v>
+        <v>0.1499758103531688</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>1ZE88F612056488798</t>
+          <t>1ZE88F611457362389</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Express</t>
         </is>
       </c>
       <c r="C17" s="7" t="n">
-        <v>19.98</v>
+        <v>35.12</v>
       </c>
       <c r="D17" s="7" t="n">
-        <v>16.98</v>
+        <v>30.27</v>
       </c>
       <c r="E17" s="8" t="n">
-        <v>3</v>
+        <v>4.85</v>
       </c>
       <c r="F17" s="9" t="n">
-        <v>0.1501501501501502</v>
+        <v>0.1380979498861048</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>1ZE88F611455999893</t>
+          <t>1ZE88F612056488798</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Express</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="C18" s="7" t="n">
-        <v>25.82</v>
+        <v>19.98</v>
       </c>
       <c r="D18" s="7" t="n">
-        <v>25.82</v>
+        <v>16.98</v>
       </c>
       <c r="E18" s="8" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F18" s="9" t="n">
-        <v>0</v>
+        <v>0.1501501501501502</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>1ZE88F611455887709</t>
+          <t>1ZE88F611455999893</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -755,190 +762,190 @@
         </is>
       </c>
       <c r="C19" s="7" t="n">
-        <v>29.76</v>
+        <v>25.82</v>
       </c>
       <c r="D19" s="7" t="n">
-        <v>25.3</v>
+        <v>25.82</v>
       </c>
       <c r="E19" s="8" t="n">
-        <v>4.46</v>
+        <v>0</v>
       </c>
       <c r="F19" s="9" t="n">
-        <v>0.1498655913978494</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>1ZE88F612056032949</t>
+          <t>1ZE88F611455887709</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Express</t>
         </is>
       </c>
       <c r="C20" s="7" t="n">
-        <v>40.73</v>
+        <v>29.76</v>
       </c>
       <c r="D20" s="7" t="n">
-        <v>34.62</v>
+        <v>25.3</v>
       </c>
       <c r="E20" s="8" t="n">
-        <v>6.11</v>
+        <v>4.46</v>
       </c>
       <c r="F20" s="9" t="n">
-        <v>0.1500122759636632</v>
+        <v>0.1498655913978494</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>1ZE88F611457542630</t>
+          <t>1ZE88F612056032949</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Express</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="C21" s="7" t="n">
-        <v>32.76</v>
+        <v>40.73</v>
       </c>
       <c r="D21" s="7" t="n">
-        <v>29.28</v>
+        <v>34.62</v>
       </c>
       <c r="E21" s="8" t="n">
-        <v>3.48</v>
+        <v>6.11</v>
       </c>
       <c r="F21" s="9" t="n">
-        <v>0.1062271062271062</v>
+        <v>0.1500122759636632</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>1ZE88F610455457111</t>
+          <t>1ZE88F611457542630</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Express Saver</t>
+          <t>Express</t>
         </is>
       </c>
       <c r="C22" s="7" t="n">
-        <v>26.32</v>
+        <v>32.76</v>
       </c>
       <c r="D22" s="7" t="n">
-        <v>26.19</v>
+        <v>29.28</v>
       </c>
       <c r="E22" s="8" t="n">
-        <v>0.13</v>
+        <v>3.48</v>
       </c>
       <c r="F22" s="9" t="n">
-        <v>0.004939209726443769</v>
+        <v>0.1062271062271062</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>1ZE88F611455973197</t>
+          <t>1ZE88F610455457111</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Express</t>
+          <t>Express Saver</t>
         </is>
       </c>
       <c r="C23" s="7" t="n">
-        <v>35.12</v>
+        <v>26.32</v>
       </c>
       <c r="D23" s="7" t="n">
-        <v>30.27</v>
+        <v>26.19</v>
       </c>
       <c r="E23" s="8" t="n">
-        <v>4.85</v>
+        <v>0.13</v>
       </c>
       <c r="F23" s="9" t="n">
-        <v>0.1380979498861048</v>
+        <v>0.004939209726443769</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>1Z5073982051446724</t>
+          <t>1ZE88F611455973197</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Standard Collect</t>
+          <t>Express</t>
         </is>
       </c>
       <c r="C24" s="7" t="n">
-        <v>57.82</v>
+        <v>35.12</v>
       </c>
       <c r="D24" s="7" t="n">
-        <v>49.15</v>
+        <v>30.27</v>
       </c>
       <c r="E24" s="8" t="n">
-        <v>8.67</v>
+        <v>4.85</v>
       </c>
       <c r="F24" s="9" t="n">
-        <v>0.149948114839156</v>
+        <v>0.1380979498861048</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>1ZE88F611456715026</t>
+          <t>1Z5073982051446724</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Express</t>
+          <t>Standard Collect</t>
         </is>
       </c>
       <c r="C25" s="7" t="n">
-        <v>35.12</v>
+        <v>57.82</v>
       </c>
       <c r="D25" s="7" t="n">
-        <v>30.27</v>
+        <v>49.15</v>
       </c>
       <c r="E25" s="8" t="n">
-        <v>4.85</v>
+        <v>8.67</v>
       </c>
       <c r="F25" s="9" t="n">
-        <v>0.1380979498861048</v>
+        <v>0.149948114839156</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>1ZE88F612055873257</t>
+          <t>1ZE88F611456715026</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Express</t>
         </is>
       </c>
       <c r="C26" s="7" t="n">
-        <v>24.2</v>
+        <v>35.12</v>
       </c>
       <c r="D26" s="7" t="n">
-        <v>20.57</v>
+        <v>30.27</v>
       </c>
       <c r="E26" s="8" t="n">
-        <v>3.63</v>
+        <v>4.85</v>
       </c>
       <c r="F26" s="9" t="n">
-        <v>0.15</v>
+        <v>0.1380979498861048</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>1ZE88F612056678761</t>
+          <t>1ZE88F612055873257</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -947,118 +954,118 @@
         </is>
       </c>
       <c r="C27" s="7" t="n">
-        <v>51.1</v>
+        <v>24.2</v>
       </c>
       <c r="D27" s="7" t="n">
-        <v>46.12</v>
+        <v>20.57</v>
       </c>
       <c r="E27" s="8" t="n">
-        <v>4.98</v>
+        <v>3.63</v>
       </c>
       <c r="F27" s="9" t="n">
-        <v>0.0974559686888454</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>1ZE88F611457673605</t>
+          <t>1ZE88F612056678761</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Express</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="C28" s="7" t="n">
-        <v>34.96</v>
+        <v>51.1</v>
       </c>
       <c r="D28" s="7" t="n">
-        <v>29.72</v>
+        <v>46.12</v>
       </c>
       <c r="E28" s="8" t="n">
-        <v>5.24</v>
+        <v>4.98</v>
       </c>
       <c r="F28" s="9" t="n">
-        <v>0.1498855835240274</v>
+        <v>0.0974559686888454</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>1ZE88F612056127427</t>
+          <t>1ZE88F611457673605</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Express</t>
         </is>
       </c>
       <c r="C29" s="7" t="n">
-        <v>39.51</v>
+        <v>34.96</v>
       </c>
       <c r="D29" s="7" t="n">
-        <v>33.58</v>
+        <v>29.72</v>
       </c>
       <c r="E29" s="8" t="n">
-        <v>5.93</v>
+        <v>5.24</v>
       </c>
       <c r="F29" s="9" t="n">
-        <v>0.1500885851683118</v>
+        <v>0.1498855835240274</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>1ZE88F611456369919</t>
+          <t>1ZE88F612056127427</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Express</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="C30" s="7" t="n">
-        <v>34.96</v>
+        <v>39.51</v>
       </c>
       <c r="D30" s="7" t="n">
-        <v>29.72</v>
+        <v>33.58</v>
       </c>
       <c r="E30" s="8" t="n">
-        <v>5.24</v>
+        <v>5.93</v>
       </c>
       <c r="F30" s="9" t="n">
-        <v>0.1498855835240274</v>
+        <v>0.1500885851683118</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>1Z5048422056773826</t>
+          <t>1ZE88F611456369919</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Standard Collect</t>
+          <t>Express</t>
         </is>
       </c>
       <c r="C31" s="7" t="n">
-        <v>40.65</v>
+        <v>34.96</v>
       </c>
       <c r="D31" s="7" t="n">
-        <v>34.55</v>
+        <v>29.72</v>
       </c>
       <c r="E31" s="8" t="n">
-        <v>6.1</v>
+        <v>5.24</v>
       </c>
       <c r="F31" s="9" t="n">
-        <v>0.1500615006150061</v>
+        <v>0.1498855835240274</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>1Z65627X2097299558</t>
+          <t>1Z5048422056773826</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1067,46 +1074,46 @@
         </is>
       </c>
       <c r="C32" s="7" t="n">
-        <v>262.74</v>
+        <v>40.65</v>
       </c>
       <c r="D32" s="7" t="n">
-        <v>223.33</v>
+        <v>34.55</v>
       </c>
       <c r="E32" s="8" t="n">
-        <v>39.41</v>
+        <v>6.1</v>
       </c>
       <c r="F32" s="9" t="n">
-        <v>0.1499961939560021</v>
+        <v>0.1500615006150061</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>1ZE88F612056338155</t>
+          <t>1Z65627X2097299558</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Standard Collect</t>
         </is>
       </c>
       <c r="C33" s="7" t="n">
-        <v>34.68</v>
+        <v>262.74</v>
       </c>
       <c r="D33" s="7" t="n">
-        <v>33.43</v>
+        <v>223.33</v>
       </c>
       <c r="E33" s="8" t="n">
-        <v>1.25</v>
+        <v>39.41</v>
       </c>
       <c r="F33" s="9" t="n">
-        <v>0.03604382929642445</v>
+        <v>0.1499961939560021</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>1ZE88F612057893517</t>
+          <t>1ZE88F612056338155</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1115,46 +1122,46 @@
         </is>
       </c>
       <c r="C34" s="7" t="n">
-        <v>25.3</v>
+        <v>34.68</v>
       </c>
       <c r="D34" s="7" t="n">
-        <v>25.01</v>
+        <v>33.43</v>
       </c>
       <c r="E34" s="8" t="n">
-        <v>0.29</v>
+        <v>1.25</v>
       </c>
       <c r="F34" s="9" t="n">
-        <v>0.01146245059288538</v>
+        <v>0.03604382929642445</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>1ZE88F611457807587</t>
+          <t>1ZE88F612057893517</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Express</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="C35" s="7" t="n">
-        <v>35.12</v>
+        <v>25.3</v>
       </c>
       <c r="D35" s="7" t="n">
-        <v>30.27</v>
+        <v>25.01</v>
       </c>
       <c r="E35" s="8" t="n">
-        <v>4.85</v>
+        <v>0.29</v>
       </c>
       <c r="F35" s="9" t="n">
-        <v>0.1380979498861048</v>
+        <v>0.01146245059288538</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>1ZE88F611457147675</t>
+          <t>1ZE88F611457807587</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1163,22 +1170,22 @@
         </is>
       </c>
       <c r="C36" s="7" t="n">
-        <v>32.88</v>
+        <v>35.12</v>
       </c>
       <c r="D36" s="7" t="n">
-        <v>29.28</v>
+        <v>30.27</v>
       </c>
       <c r="E36" s="8" t="n">
-        <v>3.6</v>
+        <v>4.85</v>
       </c>
       <c r="F36" s="9" t="n">
-        <v>0.1094890510948905</v>
+        <v>0.1380979498861048</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>1ZE88F611457504681</t>
+          <t>1ZE88F611457147675</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1187,46 +1194,46 @@
         </is>
       </c>
       <c r="C37" s="7" t="n">
-        <v>46.4</v>
+        <v>32.88</v>
       </c>
       <c r="D37" s="7" t="n">
-        <v>39.44</v>
+        <v>29.28</v>
       </c>
       <c r="E37" s="8" t="n">
-        <v>6.96</v>
+        <v>3.6</v>
       </c>
       <c r="F37" s="9" t="n">
-        <v>0.15</v>
+        <v>0.1094890510948905</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>1ZE88F612057388902</t>
+          <t>1ZE88F611457504681</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Express</t>
         </is>
       </c>
       <c r="C38" s="7" t="n">
-        <v>53.76</v>
+        <v>46.4</v>
       </c>
       <c r="D38" s="7" t="n">
-        <v>45.7</v>
+        <v>39.44</v>
       </c>
       <c r="E38" s="8" t="n">
-        <v>8.06</v>
+        <v>6.96</v>
       </c>
       <c r="F38" s="9" t="n">
-        <v>0.1499255952380953</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>1ZE88F612057606729</t>
+          <t>1ZE88F612057388902</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1235,46 +1242,46 @@
         </is>
       </c>
       <c r="C39" s="7" t="n">
-        <v>24.53</v>
+        <v>53.76</v>
       </c>
       <c r="D39" s="7" t="n">
-        <v>20.85</v>
+        <v>45.7</v>
       </c>
       <c r="E39" s="8" t="n">
-        <v>3.68</v>
+        <v>8.06</v>
       </c>
       <c r="F39" s="9" t="n">
-        <v>0.1500203832042397</v>
+        <v>0.1499255952380953</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>1ZE88F611456280737</t>
+          <t>1ZE88F612057606729</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Express</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="C40" s="7" t="n">
-        <v>35.45</v>
+        <v>24.53</v>
       </c>
       <c r="D40" s="7" t="n">
-        <v>30.27</v>
+        <v>20.85</v>
       </c>
       <c r="E40" s="8" t="n">
-        <v>5.18</v>
+        <v>3.68</v>
       </c>
       <c r="F40" s="9" t="n">
-        <v>0.1461212976022567</v>
+        <v>0.1500203832042397</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>1ZE88F611457450775</t>
+          <t>1ZE88F611456280737</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1298,7 +1305,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>1ZE88F611457633363</t>
+          <t>1ZE88F611457450775</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1307,142 +1314,142 @@
         </is>
       </c>
       <c r="C42" s="7" t="n">
-        <v>32.88</v>
+        <v>35.45</v>
       </c>
       <c r="D42" s="7" t="n">
-        <v>27.95</v>
+        <v>30.27</v>
       </c>
       <c r="E42" s="8" t="n">
-        <v>4.93</v>
+        <v>5.18</v>
       </c>
       <c r="F42" s="9" t="n">
-        <v>0.1499391727493917</v>
+        <v>0.1461212976022567</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>1ZE88F612057139127</t>
+          <t>1ZE88F611457633363</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Express</t>
         </is>
       </c>
       <c r="C43" s="7" t="n">
-        <v>58.21</v>
+        <v>32.88</v>
       </c>
       <c r="D43" s="7" t="n">
-        <v>49.48</v>
+        <v>27.95</v>
       </c>
       <c r="E43" s="8" t="n">
-        <v>8.73</v>
+        <v>4.93</v>
       </c>
       <c r="F43" s="9" t="n">
-        <v>0.1499742312317471</v>
+        <v>0.1499391727493917</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>1ZE88F611456714401</t>
+          <t>1ZE88F612057139127</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Express</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="C44" s="7" t="n">
-        <v>35.45</v>
+        <v>58.21</v>
       </c>
       <c r="D44" s="7" t="n">
-        <v>30.27</v>
+        <v>49.48</v>
       </c>
       <c r="E44" s="8" t="n">
-        <v>5.18</v>
+        <v>8.73</v>
       </c>
       <c r="F44" s="9" t="n">
-        <v>0.1461212976022567</v>
+        <v>0.1499742312317471</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>1Z65627X2090403821</t>
+          <t>1ZE88F611456714401</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Standard Collect</t>
+          <t>Express</t>
         </is>
       </c>
       <c r="C45" s="7" t="n">
-        <v>214.26</v>
+        <v>35.45</v>
       </c>
       <c r="D45" s="7" t="n">
-        <v>182.12</v>
+        <v>30.27</v>
       </c>
       <c r="E45" s="8" t="n">
-        <v>32.14</v>
+        <v>5.18</v>
       </c>
       <c r="F45" s="9" t="n">
-        <v>0.1500046672267339</v>
+        <v>0.1461212976022567</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>1ZRF7918DK95150926</t>
+          <t>1Z65627X2090403821</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Standard Third Party</t>
+          <t>Standard Collect</t>
         </is>
       </c>
       <c r="C46" s="7" t="n">
-        <v>151.56</v>
+        <v>214.26</v>
       </c>
       <c r="D46" s="7" t="n">
-        <v>128.83</v>
+        <v>182.12</v>
       </c>
       <c r="E46" s="8" t="n">
-        <v>22.73</v>
+        <v>32.14</v>
       </c>
       <c r="F46" s="9" t="n">
-        <v>0.1499736078120876</v>
+        <v>0.1500046672267339</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>1ZE88F612055341787</t>
+          <t>1ZRF7918DK95150926</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Standard Third Party</t>
         </is>
       </c>
       <c r="C47" s="7" t="n">
-        <v>30.02</v>
+        <v>151.56</v>
       </c>
       <c r="D47" s="7" t="n">
-        <v>29.01</v>
+        <v>128.83</v>
       </c>
       <c r="E47" s="8" t="n">
-        <v>1.01</v>
+        <v>22.73</v>
       </c>
       <c r="F47" s="9" t="n">
-        <v>0.03364423717521652</v>
+        <v>0.1499736078120876</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>1ZE88F612056422036</t>
+          <t>1ZE88F612055341787</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1451,22 +1458,22 @@
         </is>
       </c>
       <c r="C48" s="7" t="n">
-        <v>64.48999999999999</v>
+        <v>30.02</v>
       </c>
       <c r="D48" s="7" t="n">
-        <v>57.41</v>
+        <v>29.01</v>
       </c>
       <c r="E48" s="8" t="n">
-        <v>7.08</v>
+        <v>1.01</v>
       </c>
       <c r="F48" s="9" t="n">
-        <v>0.1097844627073965</v>
+        <v>0.03364423717521652</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>1ZE88F612055770546</t>
+          <t>1ZE88F612056422036</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1475,118 +1482,118 @@
         </is>
       </c>
       <c r="C49" s="7" t="n">
-        <v>34.41</v>
+        <v>64.48999999999999</v>
       </c>
       <c r="D49" s="7" t="n">
-        <v>34.41</v>
+        <v>57.41</v>
       </c>
       <c r="E49" s="8" t="n">
-        <v>0</v>
+        <v>7.08</v>
       </c>
       <c r="F49" s="9" t="n">
-        <v>0</v>
+        <v>0.1097844627073965</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>1ZE88F611455063170</t>
+          <t>1ZE88F612055770546</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Express</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="C50" s="7" t="n">
-        <v>32.88</v>
+        <v>34.41</v>
       </c>
       <c r="D50" s="7" t="n">
-        <v>29.28</v>
+        <v>34.41</v>
       </c>
       <c r="E50" s="8" t="n">
-        <v>3.6</v>
+        <v>0</v>
       </c>
       <c r="F50" s="9" t="n">
-        <v>0.1094890510948905</v>
+        <v>0</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>1ZE88F612057823333</t>
+          <t>1ZE88F611455063170</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Express</t>
         </is>
       </c>
       <c r="C51" s="7" t="n">
-        <v>49.75</v>
+        <v>32.88</v>
       </c>
       <c r="D51" s="7" t="n">
-        <v>48.78</v>
+        <v>29.28</v>
       </c>
       <c r="E51" s="8" t="n">
-        <v>0.97</v>
+        <v>3.6</v>
       </c>
       <c r="F51" s="9" t="n">
-        <v>0.01949748743718593</v>
+        <v>0.1094890510948905</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>1ZE88F611457958423</t>
+          <t>1ZE88F612057823333</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Express</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="C52" s="7" t="n">
-        <v>59.62</v>
+        <v>49.75</v>
       </c>
       <c r="D52" s="7" t="n">
-        <v>50.68</v>
+        <v>48.78</v>
       </c>
       <c r="E52" s="8" t="n">
-        <v>8.94</v>
+        <v>0.97</v>
       </c>
       <c r="F52" s="9" t="n">
-        <v>0.149949681314995</v>
+        <v>0.01949748743718593</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>1ZE88F612055589707</t>
+          <t>1ZE88F611457958423</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Express</t>
         </is>
       </c>
       <c r="C53" s="7" t="n">
-        <v>25.65</v>
+        <v>59.62</v>
       </c>
       <c r="D53" s="7" t="n">
-        <v>25.01</v>
+        <v>50.68</v>
       </c>
       <c r="E53" s="8" t="n">
-        <v>0.64</v>
+        <v>8.94</v>
       </c>
       <c r="F53" s="9" t="n">
-        <v>0.02495126705653022</v>
+        <v>0.149949681314995</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>1ZE88F612057457533</t>
+          <t>1ZE88F612055589707</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1595,22 +1602,22 @@
         </is>
       </c>
       <c r="C54" s="7" t="n">
-        <v>35.37</v>
+        <v>25.65</v>
       </c>
       <c r="D54" s="7" t="n">
-        <v>35.37</v>
+        <v>25.01</v>
       </c>
       <c r="E54" s="8" t="n">
-        <v>0</v>
+        <v>0.64</v>
       </c>
       <c r="F54" s="9" t="n">
-        <v>0</v>
+        <v>0.02495126705653022</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>1ZE88F612056894803</t>
+          <t>1ZE88F612057457533</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -1619,22 +1626,22 @@
         </is>
       </c>
       <c r="C55" s="7" t="n">
-        <v>35.65</v>
+        <v>35.37</v>
       </c>
       <c r="D55" s="7" t="n">
-        <v>30.3</v>
+        <v>35.37</v>
       </c>
       <c r="E55" s="8" t="n">
-        <v>5.35</v>
+        <v>0</v>
       </c>
       <c r="F55" s="9" t="n">
-        <v>0.150070126227209</v>
+        <v>0</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>1ZE88F612057484638</t>
+          <t>1ZE88F612056894803</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -1643,142 +1650,142 @@
         </is>
       </c>
       <c r="C56" s="7" t="n">
-        <v>30.21</v>
+        <v>35.65</v>
       </c>
       <c r="D56" s="7" t="n">
-        <v>30.21</v>
+        <v>30.3</v>
       </c>
       <c r="E56" s="8" t="n">
-        <v>0</v>
+        <v>5.35</v>
       </c>
       <c r="F56" s="9" t="n">
-        <v>0</v>
+        <v>0.150070126227209</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>1ZE88F611455651730</t>
+          <t>1ZE88F612057484638</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Express</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="C57" s="7" t="n">
-        <v>35.09</v>
+        <v>30.21</v>
       </c>
       <c r="D57" s="7" t="n">
-        <v>30.27</v>
+        <v>30.21</v>
       </c>
       <c r="E57" s="8" t="n">
-        <v>4.82</v>
+        <v>0</v>
       </c>
       <c r="F57" s="9" t="n">
-        <v>0.1373610715303505</v>
+        <v>0</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>1ZE88F610457637146</t>
+          <t>1ZE88F611455651730</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Express Saver</t>
+          <t>Express</t>
         </is>
       </c>
       <c r="C58" s="7" t="n">
-        <v>39.46</v>
+        <v>35.09</v>
       </c>
       <c r="D58" s="7" t="n">
-        <v>33.54</v>
+        <v>30.27</v>
       </c>
       <c r="E58" s="8" t="n">
-        <v>5.92</v>
+        <v>4.82</v>
       </c>
       <c r="F58" s="9" t="n">
-        <v>0.1500253421186011</v>
+        <v>0.1373610715303505</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>1ZE88F611456993039</t>
+          <t>1ZE88F610457637146</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Express</t>
+          <t>Express Saver</t>
         </is>
       </c>
       <c r="C59" s="7" t="n">
-        <v>46.01</v>
+        <v>39.46</v>
       </c>
       <c r="D59" s="7" t="n">
-        <v>39.11</v>
+        <v>33.54</v>
       </c>
       <c r="E59" s="8" t="n">
-        <v>6.9</v>
+        <v>5.92</v>
       </c>
       <c r="F59" s="9" t="n">
-        <v>0.149967398391654</v>
+        <v>0.1500253421186011</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>1ZE88F612055060447</t>
+          <t>1ZE88F611456993039</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Express</t>
         </is>
       </c>
       <c r="C60" s="7" t="n">
-        <v>20.9</v>
+        <v>46.01</v>
       </c>
       <c r="D60" s="7" t="n">
-        <v>17.76</v>
+        <v>39.11</v>
       </c>
       <c r="E60" s="8" t="n">
-        <v>3.14</v>
+        <v>6.9</v>
       </c>
       <c r="F60" s="9" t="n">
-        <v>0.1502392344497608</v>
+        <v>0.149967398391654</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>1ZE88F611456720136</t>
+          <t>1ZE88F612055060447</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Express</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="C61" s="7" t="n">
-        <v>59.29</v>
+        <v>20.9</v>
       </c>
       <c r="D61" s="7" t="n">
-        <v>50.4</v>
+        <v>17.76</v>
       </c>
       <c r="E61" s="8" t="n">
-        <v>8.890000000000001</v>
+        <v>3.14</v>
       </c>
       <c r="F61" s="9" t="n">
-        <v>0.1499409681227863</v>
+        <v>0.1502392344497608</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>1ZE88F611455681547</t>
+          <t>1ZE88F611456720136</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1787,22 +1794,22 @@
         </is>
       </c>
       <c r="C62" s="7" t="n">
-        <v>29.88</v>
+        <v>59.29</v>
       </c>
       <c r="D62" s="7" t="n">
-        <v>25.4</v>
+        <v>50.4</v>
       </c>
       <c r="E62" s="8" t="n">
-        <v>4.48</v>
+        <v>8.890000000000001</v>
       </c>
       <c r="F62" s="9" t="n">
-        <v>0.1499330655957162</v>
+        <v>0.1499409681227863</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>1ZE88F611455394170</t>
+          <t>1ZE88F611455681547</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -1811,22 +1818,22 @@
         </is>
       </c>
       <c r="C63" s="7" t="n">
-        <v>25.92</v>
+        <v>29.88</v>
       </c>
       <c r="D63" s="7" t="n">
-        <v>25.83</v>
+        <v>25.4</v>
       </c>
       <c r="E63" s="8" t="n">
-        <v>0.09</v>
+        <v>4.48</v>
       </c>
       <c r="F63" s="9" t="n">
-        <v>0.003472222222222222</v>
+        <v>0.1499330655957162</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>1ZE88F611455291665</t>
+          <t>1ZE88F611455394170</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1835,70 +1842,70 @@
         </is>
       </c>
       <c r="C64" s="7" t="n">
-        <v>48.99</v>
+        <v>25.92</v>
       </c>
       <c r="D64" s="7" t="n">
-        <v>41.64</v>
+        <v>25.83</v>
       </c>
       <c r="E64" s="8" t="n">
-        <v>7.35</v>
+        <v>0.09</v>
       </c>
       <c r="F64" s="9" t="n">
-        <v>0.1500306184935701</v>
+        <v>0.003472222222222222</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>1ZE88F612057740379</t>
+          <t>1ZE88F611455291665</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Express</t>
         </is>
       </c>
       <c r="C65" s="7" t="n">
-        <v>53.94</v>
+        <v>48.99</v>
       </c>
       <c r="D65" s="7" t="n">
-        <v>48.38</v>
+        <v>41.64</v>
       </c>
       <c r="E65" s="8" t="n">
-        <v>5.56</v>
+        <v>7.35</v>
       </c>
       <c r="F65" s="9" t="n">
-        <v>0.1030774935113089</v>
+        <v>0.1500306184935701</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>1ZE88F611456715651</t>
+          <t>1ZE88F612057740379</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Express</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="C66" s="7" t="n">
-        <v>35.25</v>
+        <v>53.94</v>
       </c>
       <c r="D66" s="7" t="n">
-        <v>30.27</v>
+        <v>48.38</v>
       </c>
       <c r="E66" s="8" t="n">
-        <v>4.98</v>
+        <v>5.56</v>
       </c>
       <c r="F66" s="9" t="n">
-        <v>0.1412765957446808</v>
+        <v>0.1030774935113089</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>1ZE88F611456569864</t>
+          <t>1ZE88F611456715651</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -1907,22 +1914,22 @@
         </is>
       </c>
       <c r="C67" s="7" t="n">
-        <v>32.88</v>
+        <v>35.25</v>
       </c>
       <c r="D67" s="7" t="n">
-        <v>29.28</v>
+        <v>30.27</v>
       </c>
       <c r="E67" s="8" t="n">
-        <v>3.6</v>
+        <v>4.98</v>
       </c>
       <c r="F67" s="9" t="n">
-        <v>0.1094890510948905</v>
+        <v>0.1412765957446808</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>1ZE88F611455223470</t>
+          <t>1ZE88F611456569864</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -1931,70 +1938,70 @@
         </is>
       </c>
       <c r="C68" s="7" t="n">
-        <v>39.34</v>
+        <v>32.88</v>
       </c>
       <c r="D68" s="7" t="n">
-        <v>33.44</v>
+        <v>29.28</v>
       </c>
       <c r="E68" s="8" t="n">
-        <v>5.9</v>
+        <v>3.6</v>
       </c>
       <c r="F68" s="9" t="n">
-        <v>0.1499745805795628</v>
+        <v>0.1094890510948905</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>1Z65627X0496548427</t>
+          <t>1ZE88F611455223470</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Express Saver Collect</t>
+          <t>Express</t>
         </is>
       </c>
       <c r="C69" s="7" t="n">
-        <v>101.91</v>
+        <v>39.34</v>
       </c>
       <c r="D69" s="7" t="n">
-        <v>86.62</v>
+        <v>33.44</v>
       </c>
       <c r="E69" s="8" t="n">
-        <v>15.29</v>
+        <v>5.9</v>
       </c>
       <c r="F69" s="9" t="n">
-        <v>0.1500343440290452</v>
+        <v>0.1499745805795628</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>1ZE88F612056017064</t>
+          <t>1Z65627X0496548427</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Express Saver Collect</t>
         </is>
       </c>
       <c r="C70" s="7" t="n">
-        <v>25.03</v>
+        <v>101.91</v>
       </c>
       <c r="D70" s="7" t="n">
-        <v>25.03</v>
+        <v>86.62</v>
       </c>
       <c r="E70" s="8" t="n">
-        <v>0</v>
+        <v>15.29</v>
       </c>
       <c r="F70" s="9" t="n">
-        <v>0</v>
+        <v>0.1500343440290452</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>1ZE88F612057525003</t>
+          <t>1ZE88F612056017064</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -2003,46 +2010,46 @@
         </is>
       </c>
       <c r="C71" s="7" t="n">
-        <v>42.82</v>
+        <v>25.03</v>
       </c>
       <c r="D71" s="7" t="n">
-        <v>36.4</v>
+        <v>25.03</v>
       </c>
       <c r="E71" s="8" t="n">
-        <v>6.42</v>
+        <v>0</v>
       </c>
       <c r="F71" s="9" t="n">
-        <v>0.1499299392807099</v>
+        <v>0</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>1ZE88F611455022731</t>
+          <t>1ZE88F612057525003</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Express</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="C72" s="7" t="n">
-        <v>34.99</v>
+        <v>42.82</v>
       </c>
       <c r="D72" s="7" t="n">
-        <v>30.27</v>
+        <v>36.4</v>
       </c>
       <c r="E72" s="8" t="n">
-        <v>4.72</v>
+        <v>6.42</v>
       </c>
       <c r="F72" s="9" t="n">
-        <v>0.1348956844812804</v>
+        <v>0.1499299392807099</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>1ZE88F611457290340</t>
+          <t>1ZE88F611455022731</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -2051,22 +2058,22 @@
         </is>
       </c>
       <c r="C73" s="7" t="n">
-        <v>32.64</v>
+        <v>34.99</v>
       </c>
       <c r="D73" s="7" t="n">
-        <v>27.74</v>
+        <v>30.27</v>
       </c>
       <c r="E73" s="8" t="n">
-        <v>4.9</v>
+        <v>4.72</v>
       </c>
       <c r="F73" s="9" t="n">
-        <v>0.1501225490196079</v>
+        <v>0.1348956844812804</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>1ZE88F611456177984</t>
+          <t>1ZE88F611457290340</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2078,43 +2085,43 @@
         <v>32.64</v>
       </c>
       <c r="D74" s="7" t="n">
-        <v>29.28</v>
+        <v>27.74</v>
       </c>
       <c r="E74" s="8" t="n">
-        <v>3.36</v>
+        <v>4.9</v>
       </c>
       <c r="F74" s="9" t="n">
-        <v>0.1029411764705882</v>
+        <v>0.1501225490196079</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>1Z4303702046924799</t>
+          <t>1ZE88F611456177984</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Standard Collect</t>
+          <t>Express</t>
         </is>
       </c>
       <c r="C75" s="7" t="n">
-        <v>58.82</v>
+        <v>32.64</v>
       </c>
       <c r="D75" s="7" t="n">
-        <v>50</v>
+        <v>29.28</v>
       </c>
       <c r="E75" s="8" t="n">
-        <v>8.82</v>
+        <v>3.36</v>
       </c>
       <c r="F75" s="9" t="n">
-        <v>0.1499489969398164</v>
+        <v>0.1029411764705882</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>1Z1711RE2094080962</t>
+          <t>1Z4303702046924799</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -2123,22 +2130,22 @@
         </is>
       </c>
       <c r="C76" s="7" t="n">
-        <v>59.77</v>
+        <v>58.82</v>
       </c>
       <c r="D76" s="7" t="n">
-        <v>50.8</v>
+        <v>50</v>
       </c>
       <c r="E76" s="8" t="n">
-        <v>8.970000000000001</v>
+        <v>8.82</v>
       </c>
       <c r="F76" s="9" t="n">
-        <v>0.1500752886063242</v>
+        <v>0.1499489969398164</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>1Z1711RE2094712387</t>
+          <t>1Z1711RE2094080962</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2147,22 +2154,22 @@
         </is>
       </c>
       <c r="C77" s="7" t="n">
-        <v>47.69</v>
+        <v>59.77</v>
       </c>
       <c r="D77" s="7" t="n">
-        <v>40.54</v>
+        <v>50.8</v>
       </c>
       <c r="E77" s="8" t="n">
-        <v>7.15</v>
+        <v>8.970000000000001</v>
       </c>
       <c r="F77" s="9" t="n">
-        <v>0.1499266093520654</v>
+        <v>0.1500752886063242</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>1Z4303702048875044</t>
+          <t>1Z1711RE2094712387</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2171,22 +2178,22 @@
         </is>
       </c>
       <c r="C78" s="7" t="n">
-        <v>58.46</v>
+        <v>47.69</v>
       </c>
       <c r="D78" s="7" t="n">
-        <v>49.69</v>
+        <v>40.54</v>
       </c>
       <c r="E78" s="8" t="n">
-        <v>8.77</v>
+        <v>7.15</v>
       </c>
       <c r="F78" s="9" t="n">
-        <v>0.1500171057133082</v>
+        <v>0.1499266093520654</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>1Z1711RE2092741706</t>
+          <t>1Z4303702048875044</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -2195,70 +2202,70 @@
         </is>
       </c>
       <c r="C79" s="7" t="n">
-        <v>38.85</v>
+        <v>58.46</v>
       </c>
       <c r="D79" s="7" t="n">
-        <v>33.02</v>
+        <v>49.69</v>
       </c>
       <c r="E79" s="8" t="n">
-        <v>5.83</v>
+        <v>8.77</v>
       </c>
       <c r="F79" s="9" t="n">
-        <v>0.1500643500643501</v>
+        <v>0.1500171057133082</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>1Z65627X0497694688</t>
+          <t>1Z1711RE2092741706</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Express Saver Collect</t>
+          <t>Standard Collect</t>
         </is>
       </c>
       <c r="C80" s="7" t="n">
-        <v>111.6</v>
+        <v>38.85</v>
       </c>
       <c r="D80" s="7" t="n">
-        <v>94.86</v>
+        <v>33.02</v>
       </c>
       <c r="E80" s="8" t="n">
-        <v>16.74</v>
+        <v>5.83</v>
       </c>
       <c r="F80" s="9" t="n">
-        <v>0.15</v>
+        <v>0.1500643500643501</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>1ZE88F612056729830</t>
+          <t>1Z65627X0497694688</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Express Saver Collect</t>
         </is>
       </c>
       <c r="C81" s="7" t="n">
-        <v>29.12</v>
+        <v>111.6</v>
       </c>
       <c r="D81" s="7" t="n">
-        <v>27.21</v>
+        <v>94.86</v>
       </c>
       <c r="E81" s="8" t="n">
-        <v>1.91</v>
+        <v>16.74</v>
       </c>
       <c r="F81" s="9" t="n">
-        <v>0.06559065934065933</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>1ZE88F612057347410</t>
+          <t>1ZE88F612056729830</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2282,7 +2289,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>1ZE88F612056235088</t>
+          <t>1ZE88F612057347410</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2291,46 +2298,46 @@
         </is>
       </c>
       <c r="C83" s="7" t="n">
-        <v>26.84</v>
+        <v>29.12</v>
       </c>
       <c r="D83" s="7" t="n">
-        <v>26.84</v>
+        <v>27.21</v>
       </c>
       <c r="E83" s="8" t="n">
-        <v>0</v>
+        <v>1.91</v>
       </c>
       <c r="F83" s="9" t="n">
-        <v>0</v>
+        <v>0.06559065934065933</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>1ZE88F611457566516</t>
+          <t>1ZE88F612056235088</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Express</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="C84" s="7" t="n">
-        <v>48.86</v>
+        <v>26.84</v>
       </c>
       <c r="D84" s="7" t="n">
-        <v>41.53</v>
+        <v>26.84</v>
       </c>
       <c r="E84" s="8" t="n">
-        <v>7.33</v>
+        <v>0</v>
       </c>
       <c r="F84" s="9" t="n">
-        <v>0.1500204666393778</v>
+        <v>0</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>1ZE88F611455401125</t>
+          <t>1ZE88F611457566516</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -2339,22 +2346,22 @@
         </is>
       </c>
       <c r="C85" s="7" t="n">
-        <v>43.92</v>
+        <v>48.86</v>
       </c>
       <c r="D85" s="7" t="n">
-        <v>39.91</v>
+        <v>41.53</v>
       </c>
       <c r="E85" s="8" t="n">
-        <v>4.01</v>
+        <v>7.33</v>
       </c>
       <c r="F85" s="9" t="n">
-        <v>0.09130236794171219</v>
+        <v>0.1500204666393778</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>1ZE88F611455592545</t>
+          <t>1ZE88F611455401125</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -2363,22 +2370,22 @@
         </is>
       </c>
       <c r="C86" s="7" t="n">
-        <v>55.5</v>
+        <v>43.92</v>
       </c>
       <c r="D86" s="7" t="n">
-        <v>47.18</v>
+        <v>39.91</v>
       </c>
       <c r="E86" s="8" t="n">
-        <v>8.32</v>
+        <v>4.01</v>
       </c>
       <c r="F86" s="9" t="n">
-        <v>0.1499099099099099</v>
+        <v>0.09130236794171219</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>1ZE88F611456101359</t>
+          <t>1ZE88F611455592545</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -2387,94 +2394,94 @@
         </is>
       </c>
       <c r="C87" s="7" t="n">
-        <v>52.74</v>
+        <v>55.5</v>
       </c>
       <c r="D87" s="7" t="n">
-        <v>44.83</v>
+        <v>47.18</v>
       </c>
       <c r="E87" s="8" t="n">
-        <v>7.91</v>
+        <v>8.32</v>
       </c>
       <c r="F87" s="9" t="n">
-        <v>0.1499810390595374</v>
+        <v>0.1499099099099099</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>1ZE88F612057653562</t>
+          <t>1ZE88F611456101359</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Express</t>
         </is>
       </c>
       <c r="C88" s="7" t="n">
-        <v>28.89</v>
+        <v>52.74</v>
       </c>
       <c r="D88" s="7" t="n">
-        <v>24.56</v>
+        <v>44.83</v>
       </c>
       <c r="E88" s="8" t="n">
-        <v>4.33</v>
+        <v>7.91</v>
       </c>
       <c r="F88" s="9" t="n">
-        <v>0.1498788508134302</v>
+        <v>0.1499810390595374</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>1ZE88F611455516458</t>
+          <t>1ZE88F612057653562</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Express</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="C89" s="7" t="n">
-        <v>52.56</v>
+        <v>28.89</v>
       </c>
       <c r="D89" s="7" t="n">
-        <v>44.68</v>
+        <v>24.56</v>
       </c>
       <c r="E89" s="8" t="n">
-        <v>7.88</v>
+        <v>4.33</v>
       </c>
       <c r="F89" s="9" t="n">
-        <v>0.149923896499239</v>
+        <v>0.1498788508134302</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>1ZE88F612057528279</t>
+          <t>1ZE88F611455516458</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Express</t>
         </is>
       </c>
       <c r="C90" s="7" t="n">
-        <v>26.35</v>
+        <v>52.56</v>
       </c>
       <c r="D90" s="7" t="n">
-        <v>22.4</v>
+        <v>44.68</v>
       </c>
       <c r="E90" s="8" t="n">
-        <v>3.95</v>
+        <v>7.88</v>
       </c>
       <c r="F90" s="9" t="n">
-        <v>0.1499051233396584</v>
+        <v>0.149923896499239</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>1ZE88F612056007324</t>
+          <t>1ZE88F612057528279</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -2483,22 +2490,22 @@
         </is>
       </c>
       <c r="C91" s="7" t="n">
-        <v>20.05</v>
+        <v>26.35</v>
       </c>
       <c r="D91" s="7" t="n">
-        <v>17.04</v>
+        <v>22.4</v>
       </c>
       <c r="E91" s="8" t="n">
-        <v>3.01</v>
+        <v>3.95</v>
       </c>
       <c r="F91" s="9" t="n">
-        <v>0.1501246882793017</v>
+        <v>0.1499051233396584</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>1ZE88F612055365332</t>
+          <t>1ZE88F612056007324</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -2507,22 +2514,22 @@
         </is>
       </c>
       <c r="C92" s="7" t="n">
-        <v>28.8</v>
+        <v>20.05</v>
       </c>
       <c r="D92" s="7" t="n">
-        <v>24.48</v>
+        <v>17.04</v>
       </c>
       <c r="E92" s="8" t="n">
-        <v>4.32</v>
+        <v>3.01</v>
       </c>
       <c r="F92" s="9" t="n">
-        <v>0.15</v>
+        <v>0.1501246882793017</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>1ZE88F612057246387</t>
+          <t>1ZE88F612055365332</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -2531,22 +2538,22 @@
         </is>
       </c>
       <c r="C93" s="7" t="n">
-        <v>187.75</v>
+        <v>28.8</v>
       </c>
       <c r="D93" s="7" t="n">
-        <v>159.59</v>
+        <v>24.48</v>
       </c>
       <c r="E93" s="8" t="n">
-        <v>28.16</v>
+        <v>4.32</v>
       </c>
       <c r="F93" s="9" t="n">
-        <v>0.1499866844207723</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>1ZE88F612055366653</t>
+          <t>1ZE88F612057246387</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -2555,46 +2562,46 @@
         </is>
       </c>
       <c r="C94" s="7" t="n">
-        <v>26.64</v>
+        <v>187.75</v>
       </c>
       <c r="D94" s="7" t="n">
-        <v>26.64</v>
+        <v>159.59</v>
       </c>
       <c r="E94" s="8" t="n">
-        <v>0</v>
+        <v>28.16</v>
       </c>
       <c r="F94" s="9" t="n">
-        <v>0</v>
+        <v>0.1499866844207723</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>1ZE88F611455773528</t>
+          <t>1ZE88F612055366653</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Express</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="C95" s="7" t="n">
-        <v>26.38</v>
+        <v>26.64</v>
       </c>
       <c r="D95" s="7" t="n">
-        <v>22.42</v>
+        <v>26.64</v>
       </c>
       <c r="E95" s="8" t="n">
-        <v>3.96</v>
+        <v>0</v>
       </c>
       <c r="F95" s="9" t="n">
-        <v>0.1501137225170584</v>
+        <v>0</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>1ZE88F611455599539</t>
+          <t>1ZE88F611455773528</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2603,22 +2610,22 @@
         </is>
       </c>
       <c r="C96" s="7" t="n">
-        <v>25.92</v>
+        <v>26.38</v>
       </c>
       <c r="D96" s="7" t="n">
-        <v>25.83</v>
+        <v>22.42</v>
       </c>
       <c r="E96" s="8" t="n">
-        <v>0.09</v>
+        <v>3.96</v>
       </c>
       <c r="F96" s="9" t="n">
-        <v>0.003472222222222222</v>
+        <v>0.1501137225170584</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>1ZE88F611455094995</t>
+          <t>1ZE88F611455599539</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -2627,22 +2634,22 @@
         </is>
       </c>
       <c r="C97" s="7" t="n">
-        <v>29.88</v>
+        <v>25.92</v>
       </c>
       <c r="D97" s="7" t="n">
-        <v>25.4</v>
+        <v>25.83</v>
       </c>
       <c r="E97" s="8" t="n">
-        <v>4.48</v>
+        <v>0.09</v>
       </c>
       <c r="F97" s="9" t="n">
-        <v>0.1499330655957162</v>
+        <v>0.003472222222222222</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>1ZE88F611457621116</t>
+          <t>1ZE88F611455094995</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2651,70 +2658,70 @@
         </is>
       </c>
       <c r="C98" s="7" t="n">
-        <v>53.14</v>
+        <v>29.88</v>
       </c>
       <c r="D98" s="7" t="n">
-        <v>45.17</v>
+        <v>25.4</v>
       </c>
       <c r="E98" s="8" t="n">
-        <v>7.97</v>
+        <v>4.48</v>
       </c>
       <c r="F98" s="9" t="n">
-        <v>0.1499811817839669</v>
+        <v>0.1499330655957162</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>1ZE88F612056460245</t>
+          <t>1ZE88F611457621116</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Express</t>
         </is>
       </c>
       <c r="C99" s="7" t="n">
-        <v>19.61</v>
+        <v>53.14</v>
       </c>
       <c r="D99" s="7" t="n">
-        <v>16.91</v>
+        <v>45.17</v>
       </c>
       <c r="E99" s="8" t="n">
-        <v>2.7</v>
+        <v>7.97</v>
       </c>
       <c r="F99" s="9" t="n">
-        <v>0.1376848546659868</v>
+        <v>0.1499811817839669</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>1Z65627X2090929764</t>
+          <t>1ZE88F612056460245</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Standard Collect</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="C100" s="7" t="n">
-        <v>231.52</v>
+        <v>19.61</v>
       </c>
       <c r="D100" s="7" t="n">
-        <v>196.79</v>
+        <v>16.91</v>
       </c>
       <c r="E100" s="8" t="n">
-        <v>34.73</v>
+        <v>2.7</v>
       </c>
       <c r="F100" s="9" t="n">
-        <v>0.1500086385625432</v>
+        <v>0.1376848546659868</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>1Z59296X2097993686</t>
+          <t>1Z65627X2090929764</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -2723,46 +2730,46 @@
         </is>
       </c>
       <c r="C101" s="7" t="n">
-        <v>56.69</v>
+        <v>231.52</v>
       </c>
       <c r="D101" s="7" t="n">
-        <v>48.19</v>
+        <v>196.79</v>
       </c>
       <c r="E101" s="8" t="n">
-        <v>8.5</v>
+        <v>34.73</v>
       </c>
       <c r="F101" s="9" t="n">
-        <v>0.1499382607161757</v>
+        <v>0.1500086385625432</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>1ZE88F612057271555</t>
+          <t>1Z59296X2097993686</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Standard Collect</t>
         </is>
       </c>
       <c r="C102" s="7" t="n">
-        <v>30.21</v>
+        <v>56.69</v>
       </c>
       <c r="D102" s="7" t="n">
-        <v>30.21</v>
+        <v>48.19</v>
       </c>
       <c r="E102" s="8" t="n">
-        <v>0</v>
+        <v>8.5</v>
       </c>
       <c r="F102" s="9" t="n">
-        <v>0</v>
+        <v>0.1499382607161757</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>1ZE88F612056088292</t>
+          <t>1ZE88F612057271555</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -2771,10 +2778,10 @@
         </is>
       </c>
       <c r="C103" s="7" t="n">
-        <v>47.38</v>
+        <v>30.21</v>
       </c>
       <c r="D103" s="7" t="n">
-        <v>47.38</v>
+        <v>30.21</v>
       </c>
       <c r="E103" s="8" t="n">
         <v>0</v>
@@ -2786,7 +2793,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>1ZE88F612057006369</t>
+          <t>1ZE88F612056088292</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -2795,10 +2802,10 @@
         </is>
       </c>
       <c r="C104" s="7" t="n">
-        <v>28.03</v>
+        <v>47.38</v>
       </c>
       <c r="D104" s="7" t="n">
-        <v>28.03</v>
+        <v>47.38</v>
       </c>
       <c r="E104" s="8" t="n">
         <v>0</v>
@@ -2810,55 +2817,55 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>1ZE88F611455269976</t>
+          <t>1ZE88F612057006369</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Express</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="C105" s="7" t="n">
-        <v>53.3</v>
+        <v>28.03</v>
       </c>
       <c r="D105" s="7" t="n">
-        <v>45.3</v>
+        <v>28.03</v>
       </c>
       <c r="E105" s="8" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="F105" s="9" t="n">
-        <v>0.150093808630394</v>
+        <v>0</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>1ZE88F612057048985</t>
+          <t>1ZE88F611455269976</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Express</t>
         </is>
       </c>
       <c r="C106" s="7" t="n">
-        <v>35.09</v>
+        <v>53.3</v>
       </c>
       <c r="D106" s="7" t="n">
-        <v>32.35</v>
+        <v>45.3</v>
       </c>
       <c r="E106" s="8" t="n">
-        <v>2.74</v>
+        <v>8</v>
       </c>
       <c r="F106" s="9" t="n">
-        <v>0.07808492447990881</v>
+        <v>0.150093808630394</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>1ZE88F612056838418</t>
+          <t>1ZE88F612057048985</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -2867,22 +2874,22 @@
         </is>
       </c>
       <c r="C107" s="7" t="n">
-        <v>45.23</v>
+        <v>35.09</v>
       </c>
       <c r="D107" s="7" t="n">
-        <v>40.84</v>
+        <v>32.35</v>
       </c>
       <c r="E107" s="8" t="n">
-        <v>4.39</v>
+        <v>2.74</v>
       </c>
       <c r="F107" s="9" t="n">
-        <v>0.09705947380057484</v>
+        <v>0.07808492447990881</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>1ZE88F612055639028</t>
+          <t>1ZE88F612056838418</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -2891,70 +2898,70 @@
         </is>
       </c>
       <c r="C108" s="7" t="n">
-        <v>36.89</v>
+        <v>45.23</v>
       </c>
       <c r="D108" s="7" t="n">
-        <v>31.36</v>
+        <v>40.84</v>
       </c>
       <c r="E108" s="8" t="n">
-        <v>5.53</v>
+        <v>4.39</v>
       </c>
       <c r="F108" s="9" t="n">
-        <v>0.1499051233396584</v>
+        <v>0.09705947380057484</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>1ZE88F611456552354</t>
+          <t>1ZE88F612055639028</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Express</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="C109" s="7" t="n">
-        <v>35.57</v>
+        <v>36.89</v>
       </c>
       <c r="D109" s="7" t="n">
-        <v>30.27</v>
+        <v>31.36</v>
       </c>
       <c r="E109" s="8" t="n">
-        <v>5.3</v>
+        <v>5.53</v>
       </c>
       <c r="F109" s="9" t="n">
-        <v>0.1490019679505201</v>
+        <v>0.1499051233396584</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>1ZE88F610456664645</t>
+          <t>1ZE88F611456552354</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Express Saver</t>
+          <t>Express</t>
         </is>
       </c>
       <c r="C110" s="7" t="n">
-        <v>88.47</v>
+        <v>35.57</v>
       </c>
       <c r="D110" s="7" t="n">
-        <v>75.2</v>
+        <v>30.27</v>
       </c>
       <c r="E110" s="8" t="n">
-        <v>13.27</v>
+        <v>5.3</v>
       </c>
       <c r="F110" s="9" t="n">
-        <v>0.149994348366678</v>
+        <v>0.1490019679505201</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>1ZE88F610455438329</t>
+          <t>1ZE88F610456664645</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -2963,22 +2970,22 @@
         </is>
       </c>
       <c r="C111" s="7" t="n">
-        <v>39</v>
+        <v>88.47</v>
       </c>
       <c r="D111" s="7" t="n">
-        <v>33.15</v>
+        <v>75.2</v>
       </c>
       <c r="E111" s="8" t="n">
-        <v>5.85</v>
+        <v>13.27</v>
       </c>
       <c r="F111" s="9" t="n">
-        <v>0.15</v>
+        <v>0.149994348366678</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>1ZE88F610457136339</t>
+          <t>1ZE88F610455438329</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -2987,46 +2994,46 @@
         </is>
       </c>
       <c r="C112" s="7" t="n">
-        <v>32.8</v>
+        <v>39</v>
       </c>
       <c r="D112" s="7" t="n">
-        <v>30.27</v>
+        <v>33.15</v>
       </c>
       <c r="E112" s="8" t="n">
-        <v>2.53</v>
+        <v>5.85</v>
       </c>
       <c r="F112" s="9" t="n">
-        <v>0.07713414634146341</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>1ZE88F611455242762</t>
+          <t>1ZE88F610457136339</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Express</t>
+          <t>Express Saver</t>
         </is>
       </c>
       <c r="C113" s="7" t="n">
-        <v>53.63</v>
+        <v>32.8</v>
       </c>
       <c r="D113" s="7" t="n">
-        <v>45.59</v>
+        <v>30.27</v>
       </c>
       <c r="E113" s="8" t="n">
-        <v>8.039999999999999</v>
+        <v>2.53</v>
       </c>
       <c r="F113" s="9" t="n">
-        <v>0.1499160917396979</v>
+        <v>0.07713414634146341</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>1ZE88F611455717384</t>
+          <t>1ZE88F611455242762</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -3035,70 +3042,70 @@
         </is>
       </c>
       <c r="C114" s="7" t="n">
-        <v>37.13</v>
+        <v>53.63</v>
       </c>
       <c r="D114" s="7" t="n">
-        <v>31.56</v>
+        <v>45.59</v>
       </c>
       <c r="E114" s="8" t="n">
-        <v>5.57</v>
+        <v>8.039999999999999</v>
       </c>
       <c r="F114" s="9" t="n">
-        <v>0.1500134661998384</v>
+        <v>0.1499160917396979</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>1ZE88F612056083439</t>
+          <t>1ZE88F611455717384</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Express</t>
         </is>
       </c>
       <c r="C115" s="7" t="n">
-        <v>35.02</v>
+        <v>37.13</v>
       </c>
       <c r="D115" s="7" t="n">
-        <v>35.02</v>
+        <v>31.56</v>
       </c>
       <c r="E115" s="8" t="n">
-        <v>0</v>
+        <v>5.57</v>
       </c>
       <c r="F115" s="9" t="n">
-        <v>0</v>
+        <v>0.1500134661998384</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>1ZE88F611457004524</t>
+          <t>1ZE88F612056083439</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Express</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="C116" s="7" t="n">
-        <v>33</v>
+        <v>35.02</v>
       </c>
       <c r="D116" s="7" t="n">
-        <v>30.27</v>
+        <v>35.02</v>
       </c>
       <c r="E116" s="8" t="n">
-        <v>2.73</v>
+        <v>0</v>
       </c>
       <c r="F116" s="9" t="n">
-        <v>0.08272727272727273</v>
+        <v>0</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>1ZE88F611457542952</t>
+          <t>1ZE88F611457004524</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -3107,94 +3114,94 @@
         </is>
       </c>
       <c r="C117" s="7" t="n">
-        <v>49.68</v>
+        <v>33</v>
       </c>
       <c r="D117" s="7" t="n">
-        <v>42.23</v>
+        <v>30.27</v>
       </c>
       <c r="E117" s="8" t="n">
-        <v>7.45</v>
+        <v>2.73</v>
       </c>
       <c r="F117" s="9" t="n">
-        <v>0.1499597423510467</v>
+        <v>0.08272727272727273</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>1Z5048422065523909</t>
+          <t>1ZE88F611457542952</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Standard Collect</t>
+          <t>Express</t>
         </is>
       </c>
       <c r="C118" s="7" t="n">
-        <v>41.62</v>
+        <v>49.68</v>
       </c>
       <c r="D118" s="7" t="n">
-        <v>35.38</v>
+        <v>42.23</v>
       </c>
       <c r="E118" s="8" t="n">
-        <v>6.24</v>
+        <v>7.45</v>
       </c>
       <c r="F118" s="9" t="n">
-        <v>0.1499279192695819</v>
+        <v>0.1499597423510467</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>1Z5120920498609108</t>
+          <t>1Z5048422065523909</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Express Saver Collect</t>
+          <t>Standard Collect</t>
         </is>
       </c>
       <c r="C119" s="7" t="n">
-        <v>117.87</v>
+        <v>41.62</v>
       </c>
       <c r="D119" s="7" t="n">
-        <v>100.19</v>
+        <v>35.38</v>
       </c>
       <c r="E119" s="8" t="n">
-        <v>17.68</v>
+        <v>6.24</v>
       </c>
       <c r="F119" s="9" t="n">
-        <v>0.149995758038517</v>
+        <v>0.1499279192695819</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>1ZE88F612056772695</t>
+          <t>1Z5120920498609108</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Express Saver Collect</t>
         </is>
       </c>
       <c r="C120" s="7" t="n">
-        <v>65.95</v>
+        <v>117.87</v>
       </c>
       <c r="D120" s="7" t="n">
-        <v>56.06</v>
+        <v>100.19</v>
       </c>
       <c r="E120" s="8" t="n">
-        <v>9.890000000000001</v>
+        <v>17.68</v>
       </c>
       <c r="F120" s="9" t="n">
-        <v>0.1499620924943139</v>
+        <v>0.149995758038517</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>1ZE88F612056565749</t>
+          <t>1ZE88F612056772695</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -3203,94 +3210,94 @@
         </is>
       </c>
       <c r="C121" s="7" t="n">
-        <v>31.61</v>
+        <v>65.95</v>
       </c>
       <c r="D121" s="7" t="n">
-        <v>31.48</v>
+        <v>56.06</v>
       </c>
       <c r="E121" s="8" t="n">
-        <v>0.13</v>
+        <v>9.890000000000001</v>
       </c>
       <c r="F121" s="9" t="n">
-        <v>0.004112622587788674</v>
+        <v>0.1499620924943139</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>1ZE88F611457054891</t>
+          <t>1ZE88F612056565749</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>Express</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="C122" s="7" t="n">
-        <v>103.99</v>
+        <v>31.61</v>
       </c>
       <c r="D122" s="7" t="n">
-        <v>88.39</v>
+        <v>31.48</v>
       </c>
       <c r="E122" s="8" t="n">
-        <v>15.6</v>
+        <v>0.13</v>
       </c>
       <c r="F122" s="9" t="n">
-        <v>0.1500144244638908</v>
+        <v>0.004112622587788674</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>1ZE88F612055570146</t>
+          <t>1ZE88F611457054891</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Express</t>
         </is>
       </c>
       <c r="C123" s="7" t="n">
-        <v>48.8</v>
+        <v>103.99</v>
       </c>
       <c r="D123" s="7" t="n">
-        <v>41.48</v>
+        <v>88.39</v>
       </c>
       <c r="E123" s="8" t="n">
-        <v>7.32</v>
+        <v>15.6</v>
       </c>
       <c r="F123" s="9" t="n">
-        <v>0.15</v>
+        <v>0.1500144244638908</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>1ZE88F611457625783</t>
+          <t>1ZE88F612055570146</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>Express</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="C124" s="7" t="n">
-        <v>59.84</v>
+        <v>48.8</v>
       </c>
       <c r="D124" s="7" t="n">
-        <v>50.86</v>
+        <v>41.48</v>
       </c>
       <c r="E124" s="8" t="n">
-        <v>8.98</v>
+        <v>7.32</v>
       </c>
       <c r="F124" s="9" t="n">
-        <v>0.1500668449197861</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>1ZE88F611456188267</t>
+          <t>1ZE88F611457625783</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3299,22 +3306,22 @@
         </is>
       </c>
       <c r="C125" s="7" t="n">
-        <v>37.13</v>
+        <v>59.84</v>
       </c>
       <c r="D125" s="7" t="n">
-        <v>31.56</v>
+        <v>50.86</v>
       </c>
       <c r="E125" s="8" t="n">
-        <v>5.57</v>
+        <v>8.98</v>
       </c>
       <c r="F125" s="9" t="n">
-        <v>0.1500134661998384</v>
+        <v>0.1500668449197861</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>1ZE88F611457616926</t>
+          <t>1ZE88F611456188267</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3323,22 +3330,22 @@
         </is>
       </c>
       <c r="C126" s="7" t="n">
-        <v>45.29</v>
+        <v>37.13</v>
       </c>
       <c r="D126" s="7" t="n">
-        <v>39.91</v>
+        <v>31.56</v>
       </c>
       <c r="E126" s="8" t="n">
-        <v>5.38</v>
+        <v>5.57</v>
       </c>
       <c r="F126" s="9" t="n">
-        <v>0.1187900198719364</v>
+        <v>0.1500134661998384</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>1ZE88F611457346469</t>
+          <t>1ZE88F611457616926</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -3347,190 +3354,190 @@
         </is>
       </c>
       <c r="C127" s="7" t="n">
-        <v>61.22</v>
+        <v>45.29</v>
       </c>
       <c r="D127" s="7" t="n">
-        <v>52.04</v>
+        <v>39.91</v>
       </c>
       <c r="E127" s="8" t="n">
-        <v>9.18</v>
+        <v>5.38</v>
       </c>
       <c r="F127" s="9" t="n">
-        <v>0.1499509964064031</v>
+        <v>0.1187900198719364</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>1ZE88F612055773301</t>
+          <t>1ZE88F611457346469</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Express</t>
         </is>
       </c>
       <c r="C128" s="7" t="n">
-        <v>111.43</v>
+        <v>61.22</v>
       </c>
       <c r="D128" s="7" t="n">
-        <v>94.72</v>
+        <v>52.04</v>
       </c>
       <c r="E128" s="8" t="n">
-        <v>16.71</v>
+        <v>9.18</v>
       </c>
       <c r="F128" s="9" t="n">
-        <v>0.1499596159023602</v>
+        <v>0.1499509964064031</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>1ZE88F611456774187</t>
+          <t>1ZE88F612055773301</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>Express</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="C129" s="7" t="n">
-        <v>52.85</v>
+        <v>111.43</v>
       </c>
       <c r="D129" s="7" t="n">
-        <v>44.92</v>
+        <v>94.72</v>
       </c>
       <c r="E129" s="8" t="n">
-        <v>7.93</v>
+        <v>16.71</v>
       </c>
       <c r="F129" s="9" t="n">
-        <v>0.1500473036896878</v>
+        <v>0.1499596159023602</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>1ZE88F612055264665</t>
+          <t>1ZE88F611456774187</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Express</t>
         </is>
       </c>
       <c r="C130" s="7" t="n">
-        <v>35.01</v>
+        <v>52.85</v>
       </c>
       <c r="D130" s="7" t="n">
-        <v>29.76</v>
+        <v>44.92</v>
       </c>
       <c r="E130" s="8" t="n">
-        <v>5.25</v>
+        <v>7.93</v>
       </c>
       <c r="F130" s="9" t="n">
-        <v>0.1499571550985433</v>
+        <v>0.1500473036896878</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>1ZE88F611455783697</t>
+          <t>1ZE88F612055264665</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>Express</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="C131" s="7" t="n">
-        <v>35.45</v>
+        <v>35.01</v>
       </c>
       <c r="D131" s="7" t="n">
-        <v>30.27</v>
+        <v>29.76</v>
       </c>
       <c r="E131" s="8" t="n">
-        <v>5.18</v>
+        <v>5.25</v>
       </c>
       <c r="F131" s="9" t="n">
-        <v>0.1461212976022567</v>
+        <v>0.1499571550985433</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>1ZE88F612056329414</t>
+          <t>1ZE88F611455783697</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Express</t>
         </is>
       </c>
       <c r="C132" s="7" t="n">
-        <v>56.45</v>
+        <v>35.45</v>
       </c>
       <c r="D132" s="7" t="n">
-        <v>56.45</v>
+        <v>30.27</v>
       </c>
       <c r="E132" s="8" t="n">
-        <v>0</v>
+        <v>5.18</v>
       </c>
       <c r="F132" s="9" t="n">
-        <v>0</v>
+        <v>0.1461212976022567</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>1ZE88F611455218459</t>
+          <t>1ZE88F612056329414</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>Express</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="C133" s="7" t="n">
-        <v>71.34999999999999</v>
+        <v>56.45</v>
       </c>
       <c r="D133" s="7" t="n">
-        <v>60.65</v>
+        <v>56.45</v>
       </c>
       <c r="E133" s="8" t="n">
-        <v>10.7</v>
+        <v>0</v>
       </c>
       <c r="F133" s="9" t="n">
-        <v>0.1499649614576034</v>
+        <v>0</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>1ZE88F612055276741</t>
+          <t>1ZE88F611455218459</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Express</t>
         </is>
       </c>
       <c r="C134" s="7" t="n">
-        <v>43.52</v>
+        <v>71.34999999999999</v>
       </c>
       <c r="D134" s="7" t="n">
-        <v>36.99</v>
+        <v>60.65</v>
       </c>
       <c r="E134" s="8" t="n">
-        <v>6.53</v>
+        <v>10.7</v>
       </c>
       <c r="F134" s="9" t="n">
-        <v>0.1500459558823529</v>
+        <v>0.1499649614576034</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>1ZE88F612057254430</t>
+          <t>1ZE88F612055276741</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -3539,22 +3546,22 @@
         </is>
       </c>
       <c r="C135" s="7" t="n">
-        <v>32.23</v>
+        <v>43.52</v>
       </c>
       <c r="D135" s="7" t="n">
-        <v>32.23</v>
+        <v>36.99</v>
       </c>
       <c r="E135" s="8" t="n">
-        <v>0</v>
+        <v>6.53</v>
       </c>
       <c r="F135" s="9" t="n">
-        <v>0</v>
+        <v>0.1500459558823529</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>1ZE88F612055668658</t>
+          <t>1ZE88F612057254430</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -3563,46 +3570,46 @@
         </is>
       </c>
       <c r="C136" s="7" t="n">
-        <v>58.7</v>
+        <v>32.23</v>
       </c>
       <c r="D136" s="7" t="n">
-        <v>49.9</v>
+        <v>32.23</v>
       </c>
       <c r="E136" s="8" t="n">
-        <v>8.800000000000001</v>
+        <v>0</v>
       </c>
       <c r="F136" s="9" t="n">
-        <v>0.1499148211243612</v>
+        <v>0</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>1ZE88F611456816471</t>
+          <t>1ZE88F612055668658</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>Express</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="C137" s="7" t="n">
-        <v>107.42</v>
+        <v>58.7</v>
       </c>
       <c r="D137" s="7" t="n">
-        <v>91.31</v>
+        <v>49.9</v>
       </c>
       <c r="E137" s="8" t="n">
-        <v>16.11</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="F137" s="9" t="n">
-        <v>0.1499720722398064</v>
+        <v>0.1499148211243612</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>1ZE88F611457203112</t>
+          <t>1ZE88F611456816471</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -3611,22 +3618,22 @@
         </is>
       </c>
       <c r="C138" s="7" t="n">
-        <v>33.19</v>
+        <v>107.42</v>
       </c>
       <c r="D138" s="7" t="n">
-        <v>29.28</v>
+        <v>91.31</v>
       </c>
       <c r="E138" s="8" t="n">
-        <v>3.91</v>
+        <v>16.11</v>
       </c>
       <c r="F138" s="9" t="n">
-        <v>0.1178065682434468</v>
+        <v>0.1499720722398064</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>1ZE88F611456039196</t>
+          <t>1ZE88F611457203112</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
@@ -3635,22 +3642,22 @@
         </is>
       </c>
       <c r="C139" s="7" t="n">
-        <v>26.62</v>
+        <v>33.19</v>
       </c>
       <c r="D139" s="7" t="n">
-        <v>22.63</v>
+        <v>29.28</v>
       </c>
       <c r="E139" s="8" t="n">
-        <v>3.99</v>
+        <v>3.91</v>
       </c>
       <c r="F139" s="9" t="n">
-        <v>0.1498873027798648</v>
+        <v>0.1178065682434468</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>1ZE88F611455729004</t>
+          <t>1ZE88F611456039196</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
@@ -3659,22 +3666,22 @@
         </is>
       </c>
       <c r="C140" s="7" t="n">
-        <v>250.85</v>
+        <v>26.62</v>
       </c>
       <c r="D140" s="7" t="n">
-        <v>213.22</v>
+        <v>22.63</v>
       </c>
       <c r="E140" s="8" t="n">
-        <v>37.63</v>
+        <v>3.99</v>
       </c>
       <c r="F140" s="9" t="n">
-        <v>0.1500099661152083</v>
+        <v>0.1498873027798648</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>1ZE88F611456179259</t>
+          <t>1ZE88F611455729004</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
@@ -3683,22 +3690,22 @@
         </is>
       </c>
       <c r="C141" s="7" t="n">
-        <v>53.79</v>
+        <v>250.85</v>
       </c>
       <c r="D141" s="7" t="n">
-        <v>45.72</v>
+        <v>213.22</v>
       </c>
       <c r="E141" s="8" t="n">
-        <v>8.07</v>
+        <v>37.63</v>
       </c>
       <c r="F141" s="9" t="n">
-        <v>0.1500278862242052</v>
+        <v>0.1500099661152083</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>1ZE88F611456982283</t>
+          <t>1ZE88F611456179259</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
@@ -3707,46 +3714,46 @@
         </is>
       </c>
       <c r="C142" s="7" t="n">
-        <v>39.54</v>
+        <v>53.79</v>
       </c>
       <c r="D142" s="7" t="n">
-        <v>33.61</v>
+        <v>45.72</v>
       </c>
       <c r="E142" s="8" t="n">
-        <v>5.93</v>
+        <v>8.07</v>
       </c>
       <c r="F142" s="9" t="n">
-        <v>0.1499747091552858</v>
+        <v>0.1500278862242052</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>1ZRF7918DK91426805</t>
+          <t>1ZE88F611456982283</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>Standard Collect</t>
+          <t>Express</t>
         </is>
       </c>
       <c r="C143" s="7" t="n">
-        <v>148.59</v>
+        <v>39.54</v>
       </c>
       <c r="D143" s="7" t="n">
-        <v>126.3</v>
+        <v>33.61</v>
       </c>
       <c r="E143" s="8" t="n">
-        <v>22.29</v>
+        <v>5.93</v>
       </c>
       <c r="F143" s="9" t="n">
-        <v>0.1500100948919846</v>
+        <v>0.1499747091552858</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>1Z65627X2090115419</t>
+          <t>1ZRF7918DK91426805</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
@@ -3755,22 +3762,22 @@
         </is>
       </c>
       <c r="C144" s="7" t="n">
-        <v>362.72</v>
+        <v>148.59</v>
       </c>
       <c r="D144" s="7" t="n">
-        <v>308.31</v>
+        <v>126.3</v>
       </c>
       <c r="E144" s="8" t="n">
-        <v>54.41</v>
+        <v>22.29</v>
       </c>
       <c r="F144" s="9" t="n">
-        <v>0.1500055138950154</v>
+        <v>0.1500100948919846</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>1Z65627X2098688528</t>
+          <t>1Z65627X2090115419</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -3779,22 +3786,22 @@
         </is>
       </c>
       <c r="C145" s="7" t="n">
-        <v>210.05</v>
+        <v>362.72</v>
       </c>
       <c r="D145" s="7" t="n">
-        <v>178.54</v>
+        <v>308.31</v>
       </c>
       <c r="E145" s="8" t="n">
-        <v>31.51</v>
+        <v>54.41</v>
       </c>
       <c r="F145" s="9" t="n">
-        <v>0.1500119019281123</v>
+        <v>0.1500055138950154</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>1Z65627X2098297629</t>
+          <t>1Z65627X2098688528</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -3803,22 +3810,22 @@
         </is>
       </c>
       <c r="C146" s="7" t="n">
-        <v>260.94</v>
+        <v>210.05</v>
       </c>
       <c r="D146" s="7" t="n">
-        <v>221.8</v>
+        <v>178.54</v>
       </c>
       <c r="E146" s="8" t="n">
-        <v>39.14</v>
+        <v>31.51</v>
       </c>
       <c r="F146" s="9" t="n">
-        <v>0.1499961677013873</v>
+        <v>0.1500119019281123</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>1Z65627X2093520716</t>
+          <t>1Z65627X2098297629</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
@@ -3827,47 +3834,72 @@
         </is>
       </c>
       <c r="C147" s="7" t="n">
-        <v>286.39</v>
+        <v>260.94</v>
       </c>
       <c r="D147" s="7" t="n">
-        <v>243.43</v>
+        <v>221.8</v>
       </c>
       <c r="E147" s="8" t="n">
-        <v>42.96</v>
+        <v>39.14</v>
       </c>
       <c r="F147" s="9" t="n">
-        <v>0.1500052376130452</v>
+        <v>0.1499961677013873</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
+          <t>1Z65627X2093520716</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>Standard Collect</t>
+        </is>
+      </c>
+      <c r="C148" s="7" t="n">
+        <v>286.39</v>
+      </c>
+      <c r="D148" s="7" t="n">
+        <v>243.43</v>
+      </c>
+      <c r="E148" s="8" t="n">
+        <v>42.96</v>
+      </c>
+      <c r="F148" s="9" t="n">
+        <v>0.1500052376130452</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
           <t>1Z65627X2096831072</t>
         </is>
       </c>
-      <c r="B148" t="inlineStr">
+      <c r="B149" t="inlineStr">
         <is>
           <t>Standard Collect</t>
         </is>
       </c>
-      <c r="C148" s="7" t="n">
+      <c r="C149" s="7" t="n">
         <v>62.92</v>
       </c>
-      <c r="D148" s="7" t="n">
+      <c r="D149" s="7" t="n">
         <v>53.48</v>
       </c>
-      <c r="E148" s="8" t="n">
+      <c r="E149" s="8" t="n">
         <v>9.44</v>
       </c>
-      <c r="F148" s="9" t="n">
+      <c r="F149" s="9" t="n">
         <v>0.1500317863954228</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
+    <mergeCell ref="A3:F3"/>
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>